<commit_message>
Latest code after merge withMadhukar branch
</commit_message>
<xml_diff>
--- a/Data/JTS_Approval.xlsx
+++ b/Data/JTS_Approval.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60D2F1F1-D783-4C88-BC95-9FD10C45D6C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="24">
   <si>
     <t>EmployeeID</t>
   </si>
@@ -31,49 +32,108 @@
     <t>TestStatus</t>
   </si>
   <si>
-    <t>10052303</t>
-  </si>
-  <si>
-    <t>Primary</t>
-  </si>
-  <si>
-    <t>Returns (Primary) - WFM Primary Job Transfer Sets</t>
+    <t>10283342</t>
+  </si>
+  <si>
+    <t>10196188</t>
+  </si>
+  <si>
+    <t>Secondary</t>
+  </si>
+  <si>
+    <t>Tills (Secondary) - WFM Secondary Job Transfer Sets</t>
   </si>
   <si>
     <t>Passed</t>
   </si>
   <si>
-    <t>Secondary</t>
+    <t>10493793</t>
+  </si>
+  <si>
+    <t>Fitting Rooms (Secondary) - WFM Secondary Job Transfer Sets</t>
+  </si>
+  <si>
+    <t>10513208</t>
+  </si>
+  <si>
+    <t>10513254</t>
+  </si>
+  <si>
+    <t>Zone and Maintenance (Secondary) - WFM Secondary Job Transfer Sets</t>
+  </si>
+  <si>
+    <t>10545423</t>
+  </si>
+  <si>
+    <t>SCO Host (Secondary) - WFM Secondary Job Transfer Sets</t>
+  </si>
+  <si>
+    <t>10545684</t>
+  </si>
+  <si>
+    <t>10574315</t>
   </si>
   <si>
     <t>Additional Activities (Secondary) - WFM Secondary Job Transfer Sets</t>
   </si>
   <si>
-    <t>Operations (Secondary) - WFM Secondary Job Transfer Sets</t>
+    <t>10580393</t>
+  </si>
+  <si>
+    <t>10596680</t>
+  </si>
+  <si>
+    <t>10622999</t>
+  </si>
+  <si>
+    <t>Returns (Secondary) - WFM Secondary Job Transfer Sets</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <sz val="11"/>
+      <color indexed="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -88,11 +148,23 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -115,20 +187,60 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -403,15 +515,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" customWidth="1"/>
-    <col min="4" max="4" width="57.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="28.5546875" customWidth="1"/>
+    <col min="4" max="4" width="57.44140625" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -431,89 +543,322 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>10648828</v>
-      </c>
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="3" t="s">
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>10648828</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="E2" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>10648828</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
+      <c r="E10" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="4"/>
+    </row>
+    <row r="14" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="4"/>
+    </row>
+    <row r="15" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="4"/>
+    </row>
+    <row r="16" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="4"/>
+    </row>
+    <row r="17" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="4"/>
+    </row>
+    <row r="18" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="4"/>
+    </row>
+    <row r="19" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="4"/>
+    </row>
+    <row r="20" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="4"/>
+    </row>
+    <row r="22" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="4"/>
+    </row>
+    <row r="23" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="4"/>
+    </row>
+    <row r="24" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="4"/>
+    </row>
+    <row r="25" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="4"/>
+    </row>
+    <row r="26" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="4"/>
+    </row>
+    <row r="28" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="5"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="4"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E1:E1048576">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"Failed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"Passed"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>